<commit_message>
Wrote some of the Power Block Design chapter (input filter and linear regulators)
</commit_message>
<xml_diff>
--- a/Design/Design report - calculations.xlsx
+++ b/Design/Design report - calculations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AntovI\Desktop\Projects\702\702-pumpcontrol102\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ianto\Desktop\Uni\DR_MAG\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E916F94-0DB8-4432-998E-874975B6308D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E93CE9-3407-4E9E-9CCE-C9FABCA5D2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1530" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15360" yWindow="0" windowWidth="15360" windowHeight="16680" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Voltage-Speed conversion" sheetId="1" r:id="rId1"/>
@@ -26,15 +26,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -485,13 +476,13 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1163,16 +1154,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="15.85546875" customWidth="1"/>
-    <col min="10" max="10" width="23.85546875" customWidth="1"/>
-    <col min="12" max="12" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" customWidth="1"/>
+    <col min="10" max="10" width="23.88671875" customWidth="1"/>
+    <col min="12" max="12" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1182,13 +1173,13 @@
       <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1217,7 +1208,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1243,7 +1234,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="29" t="s">
         <v>72</v>
       </c>
@@ -1260,7 +1251,7 @@
         <v>3.1625055319148934</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
         <v>70</v>
       </c>
@@ -1282,7 +1273,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="20" t="s">
         <v>71</v>
       </c>
@@ -1304,7 +1295,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>75</v>
       </c>
@@ -1325,19 +1316,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="F8" s="20"/>
       <c r="G8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="F9" s="6"/>
       <c r="G9" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="F10" s="9"/>
       <c r="G10" t="s">
         <v>64</v>
@@ -1355,16 +1346,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02AB65A6-81AD-4C02-952E-0CADC68F2ACC}">
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" customWidth="1"/>
-    <col min="12" max="12" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.109375" customWidth="1"/>
+    <col min="12" max="12" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1375,7 +1366,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>77</v>
       </c>
@@ -1398,7 +1389,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
         <v>70</v>
       </c>
@@ -1423,7 +1414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="20" t="s">
         <v>71</v>
       </c>
@@ -1443,7 +1434,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>76</v>
       </c>
@@ -1464,13 +1455,13 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="F6" s="6"/>
       <c r="G6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="F7" s="9"/>
       <c r="G7" t="s">
         <v>64</v>
@@ -1485,19 +1476,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{633E4111-6DF1-4534-9E84-DC948969C857}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" style="2"/>
-    <col min="6" max="6" width="10.28515625" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="21.5703125" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" style="2"/>
+    <col min="6" max="6" width="10.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1521,7 +1512,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1548,7 +1539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>29</v>
       </c>
@@ -1563,7 +1554,7 @@
       </c>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -1588,7 +1579,7 @@
       <c r="I4" s="5"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>79</v>
       </c>
@@ -1596,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="28">
-        <v>10</v>
+        <v>9.81</v>
       </c>
       <c r="D5" s="28">
         <v>16.62</v>
@@ -1610,7 +1601,7 @@
       <c r="I5" s="5"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>69</v>
       </c>
@@ -1620,7 +1611,7 @@
       </c>
       <c r="C6" s="35">
         <f>C4+C5</f>
-        <v>37.5</v>
+        <v>37.31</v>
       </c>
       <c r="D6" s="35">
         <f>D4+D5</f>
@@ -1632,14 +1623,14 @@
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F7" s="20"/>
       <c r="G7" t="s">
         <v>68</v>
       </c>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1657,7 +1648,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1675,7 +1666,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>33</v>
       </c>
@@ -1689,7 +1680,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
         <v>36</v>
       </c>
@@ -1706,7 +1697,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="20" t="s">
         <v>37</v>
       </c>
@@ -1722,7 +1713,7 @@
         <v>111.1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="29" t="s">
         <v>38</v>
       </c>
@@ -1739,7 +1730,7 @@
         <v>1276.4682031885482</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="20" t="s">
         <v>39</v>
       </c>
@@ -1755,7 +1746,7 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
         <v>10</v>
       </c>
@@ -1772,7 +1763,7 @@
         <v>15.889519559228651</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1789,7 +1780,7 @@
         <v>11.937557392102846</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="20" t="s">
         <v>35</v>
       </c>
@@ -1806,7 +1797,7 @@
         <v>15.832336218011145</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="20" t="s">
         <v>34</v>
       </c>
@@ -1823,7 +1814,7 @@
         <v>181.63466740821644</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>81</v>
       </c>
@@ -1833,14 +1824,14 @@
       </c>
       <c r="C20" s="3">
         <f t="shared" ref="C20:D20" si="1">C6+C16</f>
-        <v>48.86363636363636</v>
+        <v>48.673636363636362</v>
       </c>
       <c r="D20" s="3">
         <f t="shared" si="1"/>
         <v>66.688870523415986</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1857,7 +1848,7 @@
         <v>11.956436831683169</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1867,14 +1858,14 @@
       </c>
       <c r="C22" s="3">
         <f>C21*(C16+C6)/1000</f>
-        <v>0.44239359504132231</v>
+        <v>0.44067340413223144</v>
       </c>
       <c r="D22" s="3">
         <f>D21*(D16+D6)/1000</f>
         <v>0.79736126778952088</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>17</v>
       </c>
@@ -1884,22 +1875,22 @@
       </c>
       <c r="C23" s="10">
         <f>C22*$G$2+$H$2</f>
-        <v>62.119679752066119</v>
+        <v>62.033670206611575</v>
       </c>
       <c r="D23" s="10">
         <f>D22*$G$2+$H$2</f>
         <v>79.868063389476049</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -1914,19 +1905,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D89E9C3-F21D-4156-8819-A6457D9A08EB}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" style="2"/>
-    <col min="6" max="6" width="10.28515625" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="21.5703125" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" style="2"/>
+    <col min="6" max="6" width="10.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1950,7 +1941,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1980,7 +1971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>29</v>
       </c>
@@ -1995,7 +1986,7 @@
       </c>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>80</v>
       </c>
@@ -2017,7 +2008,7 @@
       <c r="I4" s="5"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>69</v>
       </c>
@@ -2042,14 +2033,14 @@
       <c r="I5" s="5"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F6" s="29"/>
       <c r="G6" t="s">
         <v>7</v>
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2068,7 +2059,7 @@
       </c>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -2086,7 +2077,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="29" t="s">
         <v>33</v>
       </c>
@@ -2104,7 +2095,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>36</v>
       </c>
@@ -2121,7 +2112,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="20" t="s">
         <v>37</v>
       </c>
@@ -2137,7 +2128,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>38</v>
       </c>
@@ -2154,7 +2145,7 @@
         <v>176.60136052156099</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="20" t="s">
         <v>39</v>
       </c>
@@ -2170,7 +2161,7 @@
         <v>166.65</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
         <v>10</v>
       </c>
@@ -2187,7 +2178,7 @@
         <v>3.5049983333333339</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2204,7 +2195,7 @@
         <v>13.131313131313133</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="20" t="s">
         <v>35</v>
       </c>
@@ -2221,7 +2212,7 @@
         <v>17.415569839812271</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="20" t="s">
         <v>34</v>
       </c>
@@ -2238,7 +2229,7 @@
         <v>32.525358534860402</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>81</v>
       </c>
@@ -2255,7 +2246,7 @@
         <v>38.131313131313135</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -2272,7 +2263,7 @@
         <v>12.747093980020731</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -2289,7 +2280,7 @@
         <v>0.48606343206644709</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
         <v>17</v>
       </c>
@@ -2306,15 +2297,15 @@
         <v>64.303171603322355</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -2329,15 +2320,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0718B513-6AED-4509-AC16-F31D3E936A65}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -2355,13 +2346,13 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="37" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
       <c r="F2" s="2">
         <v>40</v>
       </c>
@@ -2369,7 +2360,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -2385,7 +2376,7 @@
         <v>0.1515</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>48</v>
       </c>
@@ -2399,7 +2390,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -2413,7 +2404,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>52</v>
       </c>
@@ -2428,7 +2419,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -2442,7 +2433,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>50</v>
       </c>
@@ -2459,7 +2450,7 @@
         <v>0.60599999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>49</v>
       </c>
@@ -2476,15 +2467,15 @@
         <v>88.870869999999996</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="37" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="38"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -2498,7 +2489,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -2512,7 +2503,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -2526,7 +2517,7 @@
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>51</v>
       </c>
@@ -2540,7 +2531,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>52</v>
       </c>
@@ -2555,7 +2546,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>50</v>
       </c>
@@ -2571,7 +2562,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
         <v>49</v>
       </c>
@@ -2587,15 +2578,15 @@
         <v>70.264150000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="37" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>47</v>
       </c>
@@ -2609,7 +2600,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>48</v>
       </c>
@@ -2623,7 +2614,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -2637,7 +2628,7 @@
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>51</v>
       </c>
@@ -2651,7 +2642,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>52</v>
       </c>
@@ -2666,7 +2657,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -2682,7 +2673,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>49</v>
       </c>
@@ -2698,15 +2689,15 @@
         <v>73.579555555555558</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="37" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="37"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B29" s="38"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="38"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>54</v>
       </c>
@@ -2722,7 +2713,7 @@
         <v>5.0499999999999998E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>48</v>
       </c>
@@ -2736,7 +2727,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -2750,7 +2741,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>52</v>
       </c>
@@ -2765,7 +2756,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>50</v>
       </c>
@@ -2782,7 +2773,7 @@
         <v>0.505</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>49</v>
       </c>
@@ -2799,16 +2790,16 @@
         <v>114.04677272727272</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="B37" s="38"/>
-      <c r="C37" s="38">
+      <c r="B37" s="36"/>
+      <c r="C37" s="36">
         <f>5*C8+6*C17+C26+C34+'+15V power supply LM317'!$C$22+'+3.3V power supply LM317'!C21</f>
-        <v>1.6141540700413222</v>
-      </c>
-      <c r="D37" s="38"/>
+        <v>1.6124338791322312</v>
+      </c>
+      <c r="D37" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2824,16 +2815,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44971643-5616-42FB-93C8-C839C1397AF1}">
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" style="2"/>
-    <col min="6" max="6" width="10.28515625" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="10" max="10" width="21.5703125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" style="2"/>
+    <col min="6" max="6" width="10.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -2856,7 +2847,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2882,7 +2873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>29</v>
       </c>
@@ -2896,7 +2887,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -2916,7 +2907,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
         <v>62</v>
       </c>
@@ -2940,13 +2931,13 @@
       </c>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="F6" s="29"/>
       <c r="G6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2964,7 +2955,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -2982,7 +2973,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="29" t="s">
         <v>59</v>
       </c>
@@ -3000,7 +2991,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>60</v>
       </c>
@@ -3017,7 +3008,7 @@
         <v>2.5499999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="20" t="s">
         <v>23</v>
       </c>
@@ -3033,7 +3024,7 @@
         <v>4.7469999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>58</v>
       </c>
@@ -3050,7 +3041,7 @@
         <v>24.435377049180328</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="20" t="s">
         <v>22</v>
       </c>
@@ -3066,7 +3057,7 @@
         <v>23.734999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="18" t="s">
         <v>10</v>
       </c>
@@ -3083,7 +3074,7 @@
         <v>15.652515757575754</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>61</v>
       </c>
@@ -3100,7 +3091,7 @@
         <v>0.56066035380671086</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -3117,7 +3108,7 @@
         <v>11.578319158415841</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
         <v>27</v>
       </c>
@@ -3134,7 +3125,7 @@
         <v>∞</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
         <v>26</v>
       </c>
@@ -3150,7 +3141,7 @@
         <v>393.9</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -3167,7 +3158,7 @@
         <v>29.987876608173632</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="20" t="s">
         <v>24</v>
       </c>
@@ -3184,7 +3175,7 @@
         <v>0.35422353365166992</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>12</v>
       </c>
@@ -3201,7 +3192,7 @@
         <v>29.481532922983543</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -3218,7 +3209,7 @@
         <v>0.4614601586344883</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
         <v>17</v>
       </c>
@@ -3244,16 +3235,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B4CA8A-F672-402C-ABEA-CA3F1FB476B0}">
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" style="2"/>
-    <col min="6" max="6" width="10.28515625" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="10" max="10" width="21.5703125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" style="2"/>
+    <col min="6" max="6" width="10.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -3276,7 +3267,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3302,7 +3293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>29</v>
       </c>
@@ -3316,7 +3307,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -3336,7 +3327,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
         <v>62</v>
       </c>
@@ -3360,13 +3351,13 @@
       </c>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="F6" s="29"/>
       <c r="G6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -3384,7 +3375,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -3402,7 +3393,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="29" t="s">
         <v>59</v>
       </c>
@@ -3420,7 +3411,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>60</v>
       </c>
@@ -3437,7 +3428,7 @@
         <v>2.5499999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="20" t="s">
         <v>23</v>
       </c>
@@ -3453,7 +3444,7 @@
         <v>4.7469999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>58</v>
       </c>
@@ -3470,7 +3461,7 @@
         <v>1.6731229508196723</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="20" t="s">
         <v>22</v>
       </c>
@@ -3486,7 +3477,7 @@
         <v>1.5149999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="18" t="s">
         <v>10</v>
       </c>
@@ -3503,7 +3494,7 @@
         <v>3.3698897872340421</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>61</v>
       </c>
@@ -3520,7 +3511,7 @@
         <v>0.54902081903454569</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -3537,7 +3528,7 @@
         <v>22.778306595744681</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
         <v>27</v>
       </c>
@@ -3554,7 +3545,7 @@
         <v>∞</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
         <v>26</v>
       </c>
@@ -3570,7 +3561,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -3587,7 +3578,7 @@
         <v>46.016781001504405</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="20" t="s">
         <v>24</v>
       </c>
@@ -3604,7 +3595,7 @@
         <v>1.0693597875389105</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>12</v>
       </c>
@@ -3621,7 +3612,7 @@
         <v>45.502297864446703</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -3638,7 +3629,7 @@
         <v>0.15333772886908031</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
         <v>17</v>
       </c>
@@ -3664,13 +3655,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D0D6550-EC1C-4394-AF85-C4CEC96FAC1C}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" style="2"/>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -3681,7 +3672,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -3695,7 +3686,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -3709,7 +3700,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -3723,7 +3714,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -3737,7 +3728,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -3754,7 +3745,7 @@
         <v>0.17190358815543305</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -3771,7 +3762,7 @@
         <v>3.4810476601475195</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
Wrote part of the Device Configuration chapter
</commit_message>
<xml_diff>
--- a/Design/Design report - calculations.xlsx
+++ b/Design/Design report - calculations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ianto\Desktop\Uni\DR_MAG\Design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AntovI\Desktop\Uni\DR_MAG\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E93CE9-3407-4E9E-9CCE-C9FABCA5D2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4AB1208-4AF9-4E6B-AC8A-0E47A8E802B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15360" yWindow="0" windowWidth="15360" windowHeight="16680" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Voltage-Speed conversion" sheetId="1" r:id="rId1"/>
@@ -18,21 +18,31 @@
     <sheet name="+15V power supply LM317" sheetId="11" r:id="rId3"/>
     <sheet name="+3.3V power supply LM317" sheetId="12" r:id="rId4"/>
     <sheet name="Temperatures" sheetId="6" r:id="rId5"/>
-    <sheet name="(old) +15V power supply TL431" sheetId="8" r:id="rId6"/>
-    <sheet name="(old) +3.3V power supply TL431" sheetId="9" r:id="rId7"/>
-    <sheet name="(old) NTC temperature" sheetId="4" r:id="rId8"/>
+    <sheet name="Motor BEMF calculation" sheetId="13" r:id="rId6"/>
+    <sheet name="(old) +15V power supply TL431" sheetId="8" r:id="rId7"/>
+    <sheet name="(old) +3.3V power supply TL431" sheetId="9" r:id="rId8"/>
+    <sheet name="(old) NTC temperature" sheetId="4" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="99">
   <si>
     <t>Speed [RPM]</t>
   </si>
@@ -281,6 +291,54 @@
   </si>
   <si>
     <t>Ptot [W]</t>
+  </si>
+  <si>
+    <t>Back EMF constant</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Designator</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Ke</t>
+  </si>
+  <si>
+    <t>[Vrmp/kRPM]</t>
+  </si>
+  <si>
+    <t>Number of poles</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Epk</t>
+  </si>
+  <si>
+    <t>[V]</t>
+  </si>
+  <si>
+    <t>Electrical angle period of time</t>
+  </si>
+  <si>
+    <t>Peak line-to-line voltage</t>
+  </si>
+  <si>
+    <t>Telec</t>
+  </si>
+  <si>
+    <t>[ms]</t>
+  </si>
+  <si>
+    <t>Avergage:</t>
   </si>
 </sst>
 </file>
@@ -379,7 +437,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -484,6 +542,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1154,16 +1218,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="15.88671875" customWidth="1"/>
-    <col min="10" max="10" width="23.88671875" customWidth="1"/>
-    <col min="12" max="12" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="10" max="10" width="23.85546875" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1179,7 +1243,7 @@
       <c r="G1" s="37"/>
       <c r="H1" s="37"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1208,7 +1272,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1234,7 +1298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="29" t="s">
         <v>72</v>
       </c>
@@ -1251,7 +1315,7 @@
         <v>3.1625055319148934</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
         <v>70</v>
       </c>
@@ -1273,7 +1337,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
         <v>71</v>
       </c>
@@ -1295,7 +1359,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>75</v>
       </c>
@@ -1316,19 +1380,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F8" s="20"/>
       <c r="G8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F9" s="6"/>
       <c r="G9" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F10" s="9"/>
       <c r="G10" t="s">
         <v>64</v>
@@ -1346,16 +1410,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02AB65A6-81AD-4C02-952E-0CADC68F2ACC}">
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" customWidth="1"/>
-    <col min="10" max="10" width="9.109375" customWidth="1"/>
-    <col min="12" max="12" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="21.7109375" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1366,7 +1430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>77</v>
       </c>
@@ -1389,7 +1453,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>70</v>
       </c>
@@ -1414,7 +1478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>71</v>
       </c>
@@ -1434,7 +1498,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>76</v>
       </c>
@@ -1455,13 +1519,13 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="F6" s="6"/>
       <c r="G6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="F7" s="9"/>
       <c r="G7" t="s">
         <v>64</v>
@@ -1476,19 +1540,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{633E4111-6DF1-4534-9E84-DC948969C857}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" style="2"/>
-    <col min="6" max="6" width="10.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="21.5546875" customWidth="1"/>
-    <col min="11" max="11" width="9.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" style="2"/>
+    <col min="6" max="6" width="10.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1512,7 +1576,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1539,7 +1603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
         <v>29</v>
       </c>
@@ -1554,7 +1618,7 @@
       </c>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -1579,7 +1643,7 @@
       <c r="I4" s="5"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>79</v>
       </c>
@@ -1601,7 +1665,7 @@
       <c r="I5" s="5"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>69</v>
       </c>
@@ -1623,14 +1687,14 @@
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F7" s="20"/>
       <c r="G7" t="s">
         <v>68</v>
       </c>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1648,7 +1712,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1666,7 +1730,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
         <v>33</v>
       </c>
@@ -1680,7 +1744,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="29" t="s">
         <v>36</v>
       </c>
@@ -1697,7 +1761,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
         <v>37</v>
       </c>
@@ -1713,7 +1777,7 @@
         <v>111.1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="29" t="s">
         <v>38</v>
       </c>
@@ -1730,7 +1794,7 @@
         <v>1276.4682031885482</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
         <v>39</v>
       </c>
@@ -1746,7 +1810,7 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
         <v>10</v>
       </c>
@@ -1763,7 +1827,7 @@
         <v>15.889519559228651</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1780,7 +1844,7 @@
         <v>11.937557392102846</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="20" t="s">
         <v>35</v>
       </c>
@@ -1797,7 +1861,7 @@
         <v>15.832336218011145</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
         <v>34</v>
       </c>
@@ -1814,7 +1878,7 @@
         <v>181.63466740821644</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>81</v>
       </c>
@@ -1831,7 +1895,7 @@
         <v>66.688870523415986</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1848,7 +1912,7 @@
         <v>11.956436831683169</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1865,7 +1929,7 @@
         <v>0.79736126778952088</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>17</v>
       </c>
@@ -1882,15 +1946,15 @@
         <v>79.868063389476049</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -1905,19 +1969,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D89E9C3-F21D-4156-8819-A6457D9A08EB}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" style="2"/>
-    <col min="6" max="6" width="10.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="21.5546875" customWidth="1"/>
-    <col min="11" max="11" width="9.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" style="2"/>
+    <col min="6" max="6" width="10.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1941,7 +2005,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1971,7 +2035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
         <v>29</v>
       </c>
@@ -1986,7 +2050,7 @@
       </c>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>80</v>
       </c>
@@ -2008,7 +2072,7 @@
       <c r="I4" s="5"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>69</v>
       </c>
@@ -2033,14 +2097,14 @@
       <c r="I5" s="5"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F6" s="29"/>
       <c r="G6" t="s">
         <v>7</v>
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2059,7 +2123,7 @@
       </c>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -2077,7 +2141,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="29" t="s">
         <v>33</v>
       </c>
@@ -2095,7 +2159,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
         <v>36</v>
       </c>
@@ -2112,7 +2176,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>37</v>
       </c>
@@ -2128,7 +2192,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
         <v>38</v>
       </c>
@@ -2145,7 +2209,7 @@
         <v>176.60136052156099</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
         <v>39</v>
       </c>
@@ -2161,7 +2225,7 @@
         <v>166.65</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>10</v>
       </c>
@@ -2178,7 +2242,7 @@
         <v>3.5049983333333339</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2195,7 +2259,7 @@
         <v>13.131313131313133</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
         <v>35</v>
       </c>
@@ -2212,7 +2276,7 @@
         <v>17.415569839812271</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="20" t="s">
         <v>34</v>
       </c>
@@ -2229,7 +2293,7 @@
         <v>32.525358534860402</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>81</v>
       </c>
@@ -2246,7 +2310,7 @@
         <v>38.131313131313135</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -2263,7 +2327,7 @@
         <v>12.747093980020731</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -2280,7 +2344,7 @@
         <v>0.48606343206644709</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>17</v>
       </c>
@@ -2297,15 +2361,15 @@
         <v>64.303171603322355</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -2320,15 +2384,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0718B513-6AED-4509-AC16-F31D3E936A65}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -2346,7 +2410,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
         <v>74</v>
       </c>
@@ -2360,7 +2424,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -2376,7 +2440,7 @@
         <v>0.1515</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>48</v>
       </c>
@@ -2390,7 +2454,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -2404,7 +2468,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>52</v>
       </c>
@@ -2419,7 +2483,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -2433,7 +2497,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>50</v>
       </c>
@@ -2450,7 +2514,7 @@
         <v>0.60599999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>49</v>
       </c>
@@ -2467,7 +2531,7 @@
         <v>88.870869999999996</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="38" t="s">
         <v>55</v>
       </c>
@@ -2475,7 +2539,7 @@
       <c r="C11" s="38"/>
       <c r="D11" s="38"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -2489,7 +2553,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -2503,7 +2567,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -2517,7 +2581,7 @@
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>51</v>
       </c>
@@ -2531,7 +2595,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>52</v>
       </c>
@@ -2546,7 +2610,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>50</v>
       </c>
@@ -2562,7 +2626,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>49</v>
       </c>
@@ -2578,7 +2642,7 @@
         <v>70.264150000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="38" t="s">
         <v>56</v>
       </c>
@@ -2586,7 +2650,7 @@
       <c r="C20" s="38"/>
       <c r="D20" s="38"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>47</v>
       </c>
@@ -2600,7 +2664,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>48</v>
       </c>
@@ -2614,7 +2678,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -2628,7 +2692,7 @@
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>51</v>
       </c>
@@ -2642,7 +2706,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>52</v>
       </c>
@@ -2657,7 +2721,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -2673,7 +2737,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>49</v>
       </c>
@@ -2689,7 +2753,7 @@
         <v>73.579555555555558</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="38" t="s">
         <v>73</v>
       </c>
@@ -2697,7 +2761,7 @@
       <c r="C29" s="38"/>
       <c r="D29" s="38"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>54</v>
       </c>
@@ -2713,7 +2777,7 @@
         <v>5.0499999999999998E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>48</v>
       </c>
@@ -2727,7 +2791,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -2741,7 +2805,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>52</v>
       </c>
@@ -2756,7 +2820,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>50</v>
       </c>
@@ -2773,7 +2837,7 @@
         <v>0.505</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
         <v>49</v>
       </c>
@@ -2790,7 +2854,7 @@
         <v>114.04677272727272</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="s">
         <v>82</v>
       </c>
@@ -2813,438 +2877,182 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44971643-5616-42FB-93C8-C839C1397AF1}">
-  <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2271949A-1EE6-48E6-B59F-0DE58A1DEAD2}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" style="2"/>
-    <col min="6" max="6" width="10.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="10" max="10" width="21.5546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2">
         <v>8</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="26">
-        <v>22</v>
-      </c>
-      <c r="C2" s="26">
-        <v>24</v>
-      </c>
-      <c r="D2" s="26">
-        <v>26</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="2">
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="2">
+        <v>3.12</v>
+      </c>
+      <c r="E3" s="2">
+        <v>4.16</v>
+      </c>
+      <c r="F3" s="2">
+        <v>4.96</v>
+      </c>
+      <c r="G3" s="2">
+        <v>6</v>
+      </c>
+      <c r="H3" s="2">
+        <v>7.04</v>
+      </c>
+      <c r="I3" s="2">
+        <v>8</v>
+      </c>
+      <c r="J3" s="2">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="H2" s="2">
-        <v>40</v>
-      </c>
-      <c r="J2" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="25">
-        <v>15</v>
-      </c>
-      <c r="C3" s="25">
-        <v>15</v>
-      </c>
-      <c r="D3" s="25">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="28">
-        <v>0</v>
-      </c>
-      <c r="C4" s="28">
-        <v>10</v>
-      </c>
-      <c r="D4" s="27">
-        <v>16.62</v>
-      </c>
-      <c r="F4" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="29" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="13">
-        <f>B4</f>
-        <v>0</v>
-      </c>
-      <c r="C5" s="13">
-        <f>C4</f>
-        <v>10</v>
-      </c>
-      <c r="D5" s="13">
-        <f>D4</f>
-        <v>16.62</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" t="s">
-        <v>66</v>
-      </c>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="F6" s="29"/>
-      <c r="G6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2">
-        <v>2.44</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2.4950000000000001</v>
-      </c>
-      <c r="D7" s="2">
-        <v>2.5499999999999998</v>
-      </c>
-      <c r="F7" s="20"/>
-      <c r="G7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="2">
-        <v>1</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2</v>
-      </c>
-      <c r="D8" s="2">
-        <v>4</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" s="25">
-        <v>0.1</v>
-      </c>
-      <c r="C9" s="25">
-        <v>0.5</v>
-      </c>
-      <c r="D9" s="25">
-        <v>1</v>
-      </c>
-      <c r="F9" s="9"/>
-      <c r="G9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="8">
-        <f>B7/B9</f>
-        <v>24.4</v>
-      </c>
-      <c r="C10" s="13">
-        <f>C7/C9</f>
-        <v>4.99</v>
-      </c>
-      <c r="D10" s="8">
-        <f>D7/D9</f>
-        <v>2.5499999999999998</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="21">
-        <f>C11-($J$2/100*C11)</f>
-        <v>4.6530000000000005</v>
-      </c>
-      <c r="C11" s="24">
-        <v>4.7</v>
-      </c>
-      <c r="D11" s="21">
-        <f>C11+($J$2/100*C11)</f>
-        <v>4.7469999999999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="13">
-        <f>($C$3/D7-1)*B11</f>
-        <v>22.717588235294123</v>
-      </c>
-      <c r="C12" s="13">
-        <f>($C$3/C7-1)*C11</f>
-        <v>23.556513026052105</v>
-      </c>
-      <c r="D12" s="13">
-        <f>($C$3/B7-1)*D11</f>
-        <v>24.435377049180328</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="21">
-        <f>C13-($J$2/100*C13)</f>
-        <v>23.265000000000001</v>
-      </c>
-      <c r="C13" s="24">
-        <v>23.5</v>
-      </c>
-      <c r="D13" s="21">
-        <f>C13+($J$2/100*C13)</f>
-        <v>23.734999999999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="7">
-        <f>(1+B13/D11)*B7+(B8*B13)/1000</f>
-        <v>14.421680841584159</v>
-      </c>
-      <c r="C14" s="7">
-        <f>(1+C13/C11)*C7+(C8*C13)/1000</f>
-        <v>15.017000000000001</v>
-      </c>
-      <c r="D14" s="7">
-        <f>(1+D13/B11)*D7+(D8*D13)/1000</f>
-        <v>15.652515757575754</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>61</v>
-      </c>
-      <c r="B15" s="11">
-        <f>B14/(D13+D11)</f>
-        <v>0.50634368519009054</v>
-      </c>
-      <c r="C15" s="11">
-        <f>C14/(C13+C11)</f>
-        <v>0.53251773049645401</v>
-      </c>
-      <c r="D15" s="11">
-        <f>D14/(B13+B11)</f>
-        <v>0.56066035380671086</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="3">
-        <f>B2-D14</f>
-        <v>6.3474842424242457</v>
-      </c>
-      <c r="C17" s="2">
-        <f>C2-C3</f>
-        <v>9</v>
-      </c>
-      <c r="D17" s="3">
-        <f>D2-B14</f>
-        <v>11.578319158415841</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="13">
-        <f>B17/D5*1000</f>
-        <v>381.91842613864293</v>
-      </c>
-      <c r="C18" s="13">
-        <f>C17/C5*1000</f>
-        <v>900</v>
-      </c>
-      <c r="D18" s="13" t="str">
-        <f>IF(B5&lt;=0, "∞", D17/B5*1000&lt;0)</f>
-        <v>∞</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="23">
-        <f>C19-($J$2/100*C19)</f>
-        <v>386.1</v>
-      </c>
-      <c r="C19" s="24">
-        <v>390</v>
-      </c>
-      <c r="D19" s="23">
-        <f>C19+($J$2/100*C19)</f>
-        <v>393.9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="3">
-        <f>B17/D19*1000</f>
-        <v>16.114456060990722</v>
-      </c>
-      <c r="C20" s="3">
-        <f>C17/C19*1000</f>
-        <v>23.076923076923077</v>
-      </c>
-      <c r="D20" s="3">
-        <f>D17/B19*1000</f>
-        <v>29.987876608173632</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="21">
-        <f>B19*POWER(B20, 2)/1000000</f>
-        <v>0.10026078550807201</v>
-      </c>
-      <c r="C21" s="21">
-        <f>C19*POWER(C20, 2)/1000000</f>
-        <v>0.20769230769230768</v>
-      </c>
-      <c r="D21" s="21">
-        <f>D19*POWER(D20, 2)/1000000</f>
-        <v>0.35422353365166992</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B22" s="7">
-        <f>B20-D15</f>
-        <v>15.553795707184012</v>
-      </c>
-      <c r="C22" s="7">
-        <f>C20-C15</f>
-        <v>22.544405346426622</v>
-      </c>
-      <c r="D22" s="7">
-        <f>D20-B15</f>
-        <v>29.481532922983543</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24" s="3">
-        <f>B14*(IF(B22-D5&lt;0, 0, B22-D5))/1000</f>
-        <v>0</v>
-      </c>
-      <c r="C24" s="3">
-        <f>C14*(IF(C22-C5&lt;0, 0, C22-C5))/1000</f>
-        <v>0.1883793350872886</v>
-      </c>
-      <c r="D24" s="3">
-        <f>D14*(D22-B5)/1000</f>
-        <v>0.4614601586344883</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B25" s="10">
-        <f>B24*$G$2+$H$2</f>
-        <v>40</v>
-      </c>
-      <c r="C25" s="10">
-        <f>C24*$G$2+$H$2</f>
-        <v>58.272795503466995</v>
-      </c>
-      <c r="D25" s="10">
-        <f>D24*$G$2+$H$2</f>
-        <v>84.761635387545368</v>
+      <c r="D4" s="2">
+        <v>61.82</v>
+      </c>
+      <c r="E4" s="2">
+        <v>42.08</v>
+      </c>
+      <c r="F4" s="2">
+        <v>33.58</v>
+      </c>
+      <c r="G4" s="2">
+        <v>27.24</v>
+      </c>
+      <c r="H4" s="2">
+        <v>23.43</v>
+      </c>
+      <c r="I4" s="2">
+        <v>20.84</v>
+      </c>
+      <c r="J4" s="2">
+        <v>31.49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="K5" s="39" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D6" s="3">
+        <f t="shared" ref="D6:J6" si="0">D3*$D$2*D4/(120*SQRT(6))</f>
+        <v>5.2494851378270111</v>
+      </c>
+      <c r="E6" s="3">
+        <f t="shared" si="0"/>
+        <v>4.764333756060835</v>
+      </c>
+      <c r="F6" s="3">
+        <f t="shared" si="0"/>
+        <v>4.5331019243421027</v>
+      </c>
+      <c r="G6" s="3">
+        <f t="shared" si="0"/>
+        <v>4.4482733728942518</v>
+      </c>
+      <c r="H6" s="3">
+        <f t="shared" si="0"/>
+        <v>4.4892941611200614</v>
+      </c>
+      <c r="I6" s="3">
+        <f>I3*$D$2*I4/(120*SQRT(6))</f>
+        <v>4.5375436657423496</v>
+      </c>
+      <c r="J6" s="3">
+        <f>J3*$D$2*J4/(120*SQRT(6))</f>
+        <v>4.45665607112511</v>
+      </c>
+      <c r="K6" s="40">
+        <f>AVERAGE(D6:I6)</f>
+        <v>4.6703386696644351</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B4CA8A-F672-402C-ABEA-CA3F1FB476B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44971643-5616-42FB-93C8-C839C1397AF1}">
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" style="2"/>
-    <col min="6" max="6" width="10.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="10" max="10" width="21.5546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" style="2"/>
+    <col min="6" max="6" width="10.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -3267,7 +3075,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3293,21 +3101,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
         <v>29</v>
       </c>
       <c r="B3" s="25">
-        <v>3.3</v>
+        <v>15</v>
       </c>
       <c r="C3" s="25">
-        <v>3.3</v>
+        <v>15</v>
       </c>
       <c r="D3" s="25">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -3315,10 +3123,10 @@
         <v>0</v>
       </c>
       <c r="C4" s="28">
-        <v>15</v>
-      </c>
-      <c r="D4" s="28">
-        <v>25</v>
+        <v>10</v>
+      </c>
+      <c r="D4" s="27">
+        <v>16.62</v>
       </c>
       <c r="F4" s="27" t="s">
         <v>65</v>
@@ -3327,7 +3135,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="29" t="s">
         <v>62</v>
       </c>
@@ -3337,11 +3145,11 @@
       </c>
       <c r="C5" s="13">
         <f>C4</f>
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D5" s="13">
         <f>D4</f>
-        <v>25</v>
+        <v>16.62</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>65</v>
@@ -3351,13 +3159,13 @@
       </c>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F6" s="29"/>
       <c r="G6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -3375,12 +3183,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>11</v>
+      <c r="B8" s="2">
+        <v>1</v>
       </c>
       <c r="C8" s="2">
         <v>2</v>
@@ -3393,7 +3201,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="29" t="s">
         <v>59</v>
       </c>
@@ -3411,7 +3219,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
         <v>60</v>
       </c>
@@ -3428,7 +3236,7 @@
         <v>2.5499999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>23</v>
       </c>
@@ -3444,206 +3252,206 @@
         <v>4.7469999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
         <v>58</v>
       </c>
       <c r="B12" s="13">
         <f>($C$3/D7-1)*B11</f>
-        <v>1.3685294117647062</v>
+        <v>22.717588235294123</v>
       </c>
       <c r="C12" s="13">
         <f>($C$3/C7-1)*C11</f>
-        <v>1.5164328657314619</v>
+        <v>23.556513026052105</v>
       </c>
       <c r="D12" s="13">
         <f>($C$3/B7-1)*D11</f>
-        <v>1.6731229508196723</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>24.435377049180328</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
         <v>22</v>
       </c>
       <c r="B13" s="21">
         <f>C13-($J$2/100*C13)</f>
-        <v>1.4850000000000001</v>
+        <v>23.265000000000001</v>
       </c>
       <c r="C13" s="24">
-        <v>1.5</v>
+        <v>23.5</v>
       </c>
       <c r="D13" s="21">
         <f>C13+($J$2/100*C13)</f>
-        <v>1.5149999999999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>23.734999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="7">
-        <f>(1+B13/B11)*B7+(C8*B13)/1000</f>
-        <v>3.2216934042553187</v>
+        <f>(1+B13/D11)*B7+(B8*B13)/1000</f>
+        <v>14.421680841584159</v>
       </c>
       <c r="C14" s="7">
         <f>(1+C13/C11)*C7+(C8*C13)/1000</f>
-        <v>3.2942765957446807</v>
+        <v>15.017000000000001</v>
       </c>
       <c r="D14" s="7">
-        <f>(1+D13/D11)*D7+(D8*D13)/1000</f>
-        <v>3.3698897872340421</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+        <f>(1+D13/B11)*D7+(D8*D13)/1000</f>
+        <v>15.652515757575754</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>61</v>
       </c>
       <c r="B15" s="11">
         <f>B14/(D13+D11)</f>
-        <v>0.51448313705770021</v>
+        <v>0.50634368519009054</v>
       </c>
       <c r="C15" s="11">
         <f>C14/(C13+C11)</f>
-        <v>0.53133493479752913</v>
+        <v>0.53251773049645401</v>
       </c>
       <c r="D15" s="11">
         <f>D14/(B13+B11)</f>
-        <v>0.54902081903454569</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0.56066035380671086</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>25</v>
       </c>
       <c r="B17" s="3">
         <f>B2-D14</f>
-        <v>18.630110212765956</v>
+        <v>6.3474842424242457</v>
       </c>
       <c r="C17" s="2">
         <f>C2-C3</f>
-        <v>20.7</v>
+        <v>9</v>
       </c>
       <c r="D17" s="3">
         <f>D2-B14</f>
-        <v>22.778306595744681</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+        <v>11.578319158415841</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
         <v>27</v>
       </c>
       <c r="B18" s="13">
-        <f>B17/(D5*1.1)*1000</f>
-        <v>677.45855319148916</v>
+        <f>B17/D5*1000</f>
+        <v>381.91842613864293</v>
       </c>
       <c r="C18" s="13">
         <f>C17/C5*1000</f>
-        <v>1380</v>
+        <v>900</v>
       </c>
       <c r="D18" s="13" t="str">
         <f>IF(B5&lt;=0, "∞", D17/B5*1000&lt;0)</f>
         <v>∞</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="22" t="s">
         <v>26</v>
       </c>
       <c r="B19" s="23">
         <f>C19-($J$2/100*C19)</f>
-        <v>495</v>
+        <v>386.1</v>
       </c>
       <c r="C19" s="24">
-        <v>500</v>
+        <v>390</v>
       </c>
       <c r="D19" s="23">
         <f>C19+($J$2/100*C19)</f>
-        <v>505</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+        <v>393.9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>28</v>
       </c>
       <c r="B20" s="3">
         <f>B17/D19*1000</f>
-        <v>36.891307352011793</v>
+        <v>16.114456060990722</v>
       </c>
       <c r="C20" s="3">
         <f>C17/C19*1000</f>
-        <v>41.4</v>
+        <v>23.076923076923077</v>
       </c>
       <c r="D20" s="3">
         <f>D17/B19*1000</f>
-        <v>46.016781001504405</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+        <v>29.987876608173632</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="21">
         <f>B19*POWER(B20, 2)/1000000</f>
-        <v>0.67367943627959681</v>
+        <v>0.10026078550807201</v>
       </c>
       <c r="C21" s="21">
         <f>C19*POWER(C20, 2)/1000000</f>
-        <v>0.85697999999999985</v>
+        <v>0.20769230769230768</v>
       </c>
       <c r="D21" s="21">
         <f>D19*POWER(D20, 2)/1000000</f>
-        <v>1.0693597875389105</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0.35422353365166992</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B22" s="7">
         <f>B20-D15</f>
-        <v>36.342286532977248</v>
+        <v>15.553795707184012</v>
       </c>
       <c r="C22" s="7">
         <f>C20-C15</f>
-        <v>40.868665065202471</v>
+        <v>22.544405346426622</v>
       </c>
       <c r="D22" s="7">
         <f>D20-B15</f>
-        <v>45.502297864446703</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+        <v>29.481532922983543</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>13</v>
       </c>
       <c r="B24" s="3">
         <f>B14*(IF(B22-D5&lt;0, 0, B22-D5))/1000</f>
-        <v>3.6541369712466729E-2</v>
+        <v>0</v>
       </c>
       <c r="C24" s="3">
-        <f>C14*(C22-C5)/1000</f>
-        <v>8.5218537887454551E-2</v>
+        <f>C14*(IF(C22-C5&lt;0, 0, C22-C5))/1000</f>
+        <v>0.1883793350872886</v>
       </c>
       <c r="D24" s="3">
         <f>D14*(D22-B5)/1000</f>
-        <v>0.15333772886908031</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0.4614601586344883</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B25" s="10">
         <f>B24*$G$2+$H$2</f>
-        <v>43.544512862109272</v>
+        <v>40</v>
       </c>
       <c r="C25" s="10">
         <f>C24*$G$2+$H$2</f>
-        <v>48.26619817508309</v>
+        <v>58.272795503466995</v>
       </c>
       <c r="D25" s="10">
         <f>D24*$G$2+$H$2</f>
-        <v>54.873759700300795</v>
+        <v>84.761635387545368</v>
       </c>
     </row>
   </sheetData>
@@ -3653,15 +3461,435 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B4CA8A-F672-402C-ABEA-CA3F1FB476B0}">
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" style="2"/>
+    <col min="6" max="6" width="10.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="26">
+        <v>22</v>
+      </c>
+      <c r="C2" s="26">
+        <v>24</v>
+      </c>
+      <c r="D2" s="26">
+        <v>26</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="2">
+        <v>97</v>
+      </c>
+      <c r="H2" s="2">
+        <v>40</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="25">
+        <v>3.3</v>
+      </c>
+      <c r="C3" s="25">
+        <v>3.3</v>
+      </c>
+      <c r="D3" s="25">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="28">
+        <v>0</v>
+      </c>
+      <c r="C4" s="28">
+        <v>15</v>
+      </c>
+      <c r="D4" s="28">
+        <v>25</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="13">
+        <f>B4</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="13">
+        <f>C4</f>
+        <v>15</v>
+      </c>
+      <c r="D5" s="13">
+        <f>D4</f>
+        <v>25</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" t="s">
+        <v>66</v>
+      </c>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F6" s="29"/>
+      <c r="G6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2">
+        <v>2.44</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2.4950000000000001</v>
+      </c>
+      <c r="D7" s="2">
+        <v>2.5499999999999998</v>
+      </c>
+      <c r="F7" s="20"/>
+      <c r="G7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2</v>
+      </c>
+      <c r="D8" s="2">
+        <v>4</v>
+      </c>
+      <c r="F8" s="6"/>
+      <c r="G8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="C9" s="25">
+        <v>0.5</v>
+      </c>
+      <c r="D9" s="25">
+        <v>1</v>
+      </c>
+      <c r="F9" s="9"/>
+      <c r="G9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="8">
+        <f>B7/B9</f>
+        <v>24.4</v>
+      </c>
+      <c r="C10" s="13">
+        <f>C7/C9</f>
+        <v>4.99</v>
+      </c>
+      <c r="D10" s="8">
+        <f>D7/D9</f>
+        <v>2.5499999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="21">
+        <f>C11-($J$2/100*C11)</f>
+        <v>4.6530000000000005</v>
+      </c>
+      <c r="C11" s="24">
+        <v>4.7</v>
+      </c>
+      <c r="D11" s="21">
+        <f>C11+($J$2/100*C11)</f>
+        <v>4.7469999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="13">
+        <f>($C$3/D7-1)*B11</f>
+        <v>1.3685294117647062</v>
+      </c>
+      <c r="C12" s="13">
+        <f>($C$3/C7-1)*C11</f>
+        <v>1.5164328657314619</v>
+      </c>
+      <c r="D12" s="13">
+        <f>($C$3/B7-1)*D11</f>
+        <v>1.6731229508196723</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="21">
+        <f>C13-($J$2/100*C13)</f>
+        <v>1.4850000000000001</v>
+      </c>
+      <c r="C13" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="D13" s="21">
+        <f>C13+($J$2/100*C13)</f>
+        <v>1.5149999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="7">
+        <f>(1+B13/B11)*B7+(C8*B13)/1000</f>
+        <v>3.2216934042553187</v>
+      </c>
+      <c r="C14" s="7">
+        <f>(1+C13/C11)*C7+(C8*C13)/1000</f>
+        <v>3.2942765957446807</v>
+      </c>
+      <c r="D14" s="7">
+        <f>(1+D13/D11)*D7+(D8*D13)/1000</f>
+        <v>3.3698897872340421</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="11">
+        <f>B14/(D13+D11)</f>
+        <v>0.51448313705770021</v>
+      </c>
+      <c r="C15" s="11">
+        <f>C14/(C13+C11)</f>
+        <v>0.53133493479752913</v>
+      </c>
+      <c r="D15" s="11">
+        <f>D14/(B13+B11)</f>
+        <v>0.54902081903454569</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="3">
+        <f>B2-D14</f>
+        <v>18.630110212765956</v>
+      </c>
+      <c r="C17" s="2">
+        <f>C2-C3</f>
+        <v>20.7</v>
+      </c>
+      <c r="D17" s="3">
+        <f>D2-B14</f>
+        <v>22.778306595744681</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="13">
+        <f>B17/(D5*1.1)*1000</f>
+        <v>677.45855319148916</v>
+      </c>
+      <c r="C18" s="13">
+        <f>C17/C5*1000</f>
+        <v>1380</v>
+      </c>
+      <c r="D18" s="13" t="str">
+        <f>IF(B5&lt;=0, "∞", D17/B5*1000&lt;0)</f>
+        <v>∞</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="23">
+        <f>C19-($J$2/100*C19)</f>
+        <v>495</v>
+      </c>
+      <c r="C19" s="24">
+        <v>500</v>
+      </c>
+      <c r="D19" s="23">
+        <f>C19+($J$2/100*C19)</f>
+        <v>505</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="3">
+        <f>B17/D19*1000</f>
+        <v>36.891307352011793</v>
+      </c>
+      <c r="C20" s="3">
+        <f>C17/C19*1000</f>
+        <v>41.4</v>
+      </c>
+      <c r="D20" s="3">
+        <f>D17/B19*1000</f>
+        <v>46.016781001504405</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="21">
+        <f>B19*POWER(B20, 2)/1000000</f>
+        <v>0.67367943627959681</v>
+      </c>
+      <c r="C21" s="21">
+        <f>C19*POWER(C20, 2)/1000000</f>
+        <v>0.85697999999999985</v>
+      </c>
+      <c r="D21" s="21">
+        <f>D19*POWER(D20, 2)/1000000</f>
+        <v>1.0693597875389105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" s="7">
+        <f>B20-D15</f>
+        <v>36.342286532977248</v>
+      </c>
+      <c r="C22" s="7">
+        <f>C20-C15</f>
+        <v>40.868665065202471</v>
+      </c>
+      <c r="D22" s="7">
+        <f>D20-B15</f>
+        <v>45.502297864446703</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" s="3">
+        <f>B14*(IF(B22-D5&lt;0, 0, B22-D5))/1000</f>
+        <v>3.6541369712466729E-2</v>
+      </c>
+      <c r="C24" s="3">
+        <f>C14*(C22-C5)/1000</f>
+        <v>8.5218537887454551E-2</v>
+      </c>
+      <c r="D24" s="3">
+        <f>D14*(D22-B5)/1000</f>
+        <v>0.15333772886908031</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="10">
+        <f>B24*$G$2+$H$2</f>
+        <v>43.544512862109272</v>
+      </c>
+      <c r="C25" s="10">
+        <f>C24*$G$2+$H$2</f>
+        <v>48.26619817508309</v>
+      </c>
+      <c r="D25" s="10">
+        <f>D24*$G$2+$H$2</f>
+        <v>54.873759700300795</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D0D6550-EC1C-4394-AF85-C4CEC96FAC1C}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" style="2"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -3672,7 +3900,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -3686,7 +3914,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -3700,7 +3928,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -3714,7 +3942,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -3728,7 +3956,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -3745,7 +3973,7 @@
         <v>0.17190358815543305</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -3762,7 +3990,7 @@
         <v>3.4810476601475195</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>45</v>
       </c>

</xml_diff>